<commit_message>
Adapting VGG16 to the GAN
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sluedu-my.sharepoint.com/personal/felipe_lopes_slu_edu/Documents/Desktop/Repos/plant-disease-prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="386" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{184BE264-263A-43B4-99BE-B039D3215C5D}"/>
+  <xr:revisionPtr revIDLastSave="388" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CD19BF6-5830-498E-91B5-F75C5AE76B10}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1259,16 +1259,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>323850</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>

<commit_message>
- Changing the GAN to use VGG16 - Verifying the feature extraction to solve the index problem
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sluedu-my.sharepoint.com/personal/felipe_lopes_slu_edu/Documents/Desktop/Repos/plant-disease-prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="388" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CD19BF6-5830-498E-91B5-F75C5AE76B10}"/>
+  <xr:revisionPtr revIDLastSave="389" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92FB6E64-2531-4743-8A30-E35E22D2DC80}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1259,15 +1259,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>323850</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1238250</xdr:colOff>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">

</xml_diff>

<commit_message>
Updating feature extraction code and results.
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sluedu-my.sharepoint.com/personal/felipe_lopes_slu_edu/Documents/Desktop/Repos/plant-disease-prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="392" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D986AA2-0296-4720-850E-B1B9381BC66C}"/>
+  <xr:revisionPtr revIDLastSave="424" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70C72321-DD0E-4E67-A365-B1B3319C9481}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall Analysis" sheetId="1" r:id="rId1"/>
-    <sheet name="08-30 Analysis" sheetId="2" r:id="rId2"/>
-    <sheet name="Three first days Analaysis" sheetId="4" r:id="rId3"/>
-    <sheet name="All but last Analysis" sheetId="3" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId2"/>
+    <sheet name="08-30 Analysis" sheetId="2" r:id="rId3"/>
+    <sheet name="Three first days Analaysis" sheetId="4" r:id="rId4"/>
+    <sheet name="All but last Analysis" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="36">
   <si>
     <t>SVM</t>
   </si>
@@ -141,14 +142,28 @@
   </si>
   <si>
     <t>ARI_2</t>
+  </si>
+  <si>
+    <t>OVERSAMPLED</t>
+  </si>
+  <si>
+    <t>UNBALANCED</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -176,10 +191,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -223,7 +239,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'08-30 Analysis'!$A$3</c:f>
+              <c:f>'08-30 Analysis'!$A$20</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -244,7 +260,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'08-30 Analysis'!$B$1:$H$2</c:f>
+              <c:f>'08-30 Analysis'!$B$1:$H$19</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="7"/>
                 <c:lvl>
@@ -283,7 +299,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'08-30 Analysis'!$B$3:$H$3</c:f>
+              <c:f>'08-30 Analysis'!$B$20:$H$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -322,7 +338,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'08-30 Analysis'!$A$4</c:f>
+              <c:f>'08-30 Analysis'!$A$21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -343,7 +359,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'08-30 Analysis'!$B$1:$H$2</c:f>
+              <c:f>'08-30 Analysis'!$B$1:$H$19</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="7"/>
                 <c:lvl>
@@ -382,7 +398,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'08-30 Analysis'!$B$4:$H$4</c:f>
+              <c:f>'08-30 Analysis'!$B$21:$H$21</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -421,7 +437,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'08-30 Analysis'!$A$5</c:f>
+              <c:f>'08-30 Analysis'!$A$22</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -442,7 +458,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'08-30 Analysis'!$B$1:$H$2</c:f>
+              <c:f>'08-30 Analysis'!$B$1:$H$19</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="7"/>
                 <c:lvl>
@@ -481,7 +497,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'08-30 Analysis'!$B$5:$H$5</c:f>
+              <c:f>'08-30 Analysis'!$B$22:$H$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1261,13 +1277,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1238250</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>295275</xdr:colOff>
-      <xdr:row>45</xdr:row>
+      <xdr:row>56</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1294,6 +1310,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1987,8 +2007,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31B271D7-5147-414E-9D6E-4A27129EAAD6}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D5AA18C-A5F0-4069-B351-4AEFF0D48C38}">
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
@@ -2037,332 +2066,461 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>9</v>
       </c>
-      <c r="B3">
+      <c r="B20">
         <v>0.26</v>
       </c>
-      <c r="C3">
+      <c r="C20">
         <v>0.35</v>
       </c>
-      <c r="D3">
+      <c r="D20">
         <v>0.36</v>
       </c>
-      <c r="E3">
+      <c r="E20">
         <v>0.88</v>
       </c>
-      <c r="F3">
+      <c r="F20">
         <v>0.33</v>
       </c>
-      <c r="G3">
+      <c r="G20">
         <v>0.96</v>
       </c>
-      <c r="H3">
+      <c r="H20">
         <v>0.96</v>
       </c>
-      <c r="I3">
+      <c r="I20">
         <v>0.9</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>10</v>
       </c>
-      <c r="B4">
+      <c r="B21">
         <v>0.24</v>
       </c>
-      <c r="C4">
+      <c r="C21">
         <v>0.16</v>
       </c>
-      <c r="D4">
+      <c r="D21">
         <v>0.55000000000000004</v>
       </c>
-      <c r="E4">
+      <c r="E21">
         <v>0.57999999999999996</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0.93</v>
-      </c>
-      <c r="H4">
-        <v>0.95</v>
-      </c>
-      <c r="I4">
-        <v>0.93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0.78</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0.9</v>
-      </c>
-      <c r="H5">
-        <v>0.87</v>
-      </c>
-      <c r="I5">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="C6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="E6">
-        <v>0.38</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>1.96</v>
-      </c>
-      <c r="C7">
-        <v>1.88</v>
-      </c>
-      <c r="E7">
-        <v>0.53</v>
-      </c>
-      <c r="F7">
-        <v>1.66</v>
-      </c>
-      <c r="I7">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8">
-        <v>-1.29</v>
-      </c>
-      <c r="C8">
-        <v>-0.98</v>
-      </c>
-      <c r="E8">
-        <v>-0.26</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9">
-        <v>0.25</v>
-      </c>
-      <c r="C9">
-        <v>0.27</v>
-      </c>
-      <c r="E9">
-        <v>0.68</v>
-      </c>
-      <c r="F9">
-        <v>0.33</v>
-      </c>
-      <c r="I9">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10">
-        <v>0.25</v>
-      </c>
-      <c r="C10">
-        <v>0.27</v>
-      </c>
-      <c r="E10">
-        <v>0.68</v>
-      </c>
-      <c r="F10">
-        <v>0.25</v>
-      </c>
-      <c r="I10">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F16">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>22</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>24</v>
-      </c>
-      <c r="F19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>25</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>26</v>
       </c>
       <c r="F21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G21">
+        <v>0.93</v>
+      </c>
+      <c r="H21">
+        <v>0.95</v>
+      </c>
+      <c r="I21">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0.78</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>0.9</v>
+      </c>
+      <c r="H22">
+        <v>0.87</v>
+      </c>
+      <c r="I22">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="C23">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E23">
+        <v>0.38</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24">
+        <v>1.96</v>
+      </c>
+      <c r="C24">
+        <v>1.88</v>
+      </c>
+      <c r="E24">
+        <v>0.53</v>
+      </c>
+      <c r="F24">
+        <v>1.66</v>
+      </c>
+      <c r="I24">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25">
+        <v>-1.29</v>
+      </c>
+      <c r="C25">
+        <v>-0.98</v>
+      </c>
+      <c r="E25">
+        <v>-0.26</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26">
+        <v>0.25</v>
+      </c>
+      <c r="C26">
+        <v>0.27</v>
+      </c>
+      <c r="E26">
+        <v>0.68</v>
+      </c>
+      <c r="F26">
+        <v>0.33</v>
+      </c>
+      <c r="I26">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27">
+        <v>0.25</v>
+      </c>
+      <c r="C27">
+        <v>0.27</v>
+      </c>
+      <c r="E27">
+        <v>0.68</v>
+      </c>
+      <c r="F27">
+        <v>0.25</v>
+      </c>
+      <c r="I27">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>27</v>
       </c>
-      <c r="F22">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>28</v>
       </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>29</v>
       </c>
-      <c r="F24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>30</v>
       </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>31</v>
       </c>
-      <c r="F26">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>32</v>
       </c>
-      <c r="F27">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>33</v>
-      </c>
-      <c r="F28">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA01A254-30FA-4066-BC2B-BE8C98A6CE0D}">
   <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2561,7 +2719,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04300482-AF1D-4DE0-B0C9-9A57AF676E66}">
   <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Changes to the training phase.
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26501"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sluedu-my.sharepoint.com/personal/felipe_lopes_slu_edu/Documents/Desktop/Repos/plant-disease-prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="424" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70C72321-DD0E-4E67-A365-B1B3319C9481}"/>
+  <xr:revisionPtr revIDLastSave="508" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5390C6E-E83E-4D55-8EAB-F63804077374}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall Analysis" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="5" r:id="rId2"/>
-    <sheet name="08-30 Analysis" sheetId="2" r:id="rId3"/>
-    <sheet name="Three first days Analaysis" sheetId="4" r:id="rId4"/>
-    <sheet name="All but last Analysis" sheetId="3" r:id="rId5"/>
+    <sheet name="08-30 Analysis" sheetId="2" r:id="rId2"/>
+    <sheet name="Three first days Analaysis" sheetId="4" r:id="rId3"/>
+    <sheet name="All but last Analysis" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +39,22 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="33">
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>Samples</t>
+  </si>
+  <si>
+    <t>Mild</t>
+  </si>
+  <si>
+    <t>Unhealthy</t>
+  </si>
+  <si>
+    <t>Healthy</t>
+  </si>
   <si>
     <t>SVM</t>
   </si>
@@ -48,34 +62,7 @@
     <t>RFO</t>
   </si>
   <si>
-    <t>ARIMA</t>
-  </si>
-  <si>
-    <t>8/30/2021 Unbalanced</t>
-  </si>
-  <si>
-    <t>8/30/2021 Balanced Test</t>
-  </si>
-  <si>
-    <t>8/30/2021 Balanced Validation</t>
-  </si>
-  <si>
-    <t>All Dates Unbalanced</t>
-  </si>
-  <si>
-    <t>All Dates Balanced Test</t>
-  </si>
-  <si>
-    <t>All Dates Balanced Validation</t>
-  </si>
-  <si>
-    <t>Healthy</t>
-  </si>
-  <si>
-    <t>Unhealthy</t>
-  </si>
-  <si>
-    <t>Mild</t>
+    <t>SYNTHETICALLY BALANCED</t>
   </si>
   <si>
     <t>MAE</t>
@@ -91,6 +78,12 @@
   </si>
   <si>
     <t>Accuracy</t>
+  </si>
+  <si>
+    <t>UNBALANCED</t>
+  </si>
+  <si>
+    <t>OVERSAMPLED</t>
   </si>
   <si>
     <t>Feature Importance</t>
@@ -144,17 +137,14 @@
     <t>ARI_2</t>
   </si>
   <si>
-    <t>OVERSAMPLED</t>
-  </si>
-  <si>
-    <t>UNBALANCED</t>
+    <t>ARIMA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -216,7 +206,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="pt-BR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -227,7 +217,391 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Dataset distribution</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Crop label</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Overall Analysis'!$A$2:$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Mild</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Unhealthy</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Healthy</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Overall Analysis'!$B$2:$B$4</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>205</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-4C24-468F-939B-EC3C370ED38C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="822061416"/>
+        <c:axId val="1154371576"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="822061416"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1154371576"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1154371576"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="822061416"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Oversampled Dataset</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
@@ -239,7 +613,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'08-30 Analysis'!$A$20</c:f>
+              <c:f>'08-30 Analysis'!$A$22</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -258,48 +632,9 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:multiLvlStrRef>
-              <c:f>'08-30 Analysis'!$B$1:$H$19</c:f>
-              <c:multiLvlStrCache>
-                <c:ptCount val="7"/>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>24-Sep</c:v>
-                  </c:pt>
-                  <c:pt idx="1">
-                    <c:v>5-Oct</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>26-Oct</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>17-Nov</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>24-Sep</c:v>
-                  </c:pt>
-                  <c:pt idx="5">
-                    <c:v>5-Oct</c:v>
-                  </c:pt>
-                  <c:pt idx="6">
-                    <c:v>26-Oct</c:v>
-                  </c:pt>
-                </c:lvl>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>SVM</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>RFO</c:v>
-                  </c:pt>
-                </c:lvl>
-              </c:multiLvlStrCache>
-            </c:multiLvlStrRef>
-          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'08-30 Analysis'!$B$20:$H$20</c:f>
+              <c:f>'08-30 Analysis'!$B$22:$H$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -338,7 +673,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'08-30 Analysis'!$A$21</c:f>
+              <c:f>'08-30 Analysis'!$A$23</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -357,48 +692,9 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:multiLvlStrRef>
-              <c:f>'08-30 Analysis'!$B$1:$H$19</c:f>
-              <c:multiLvlStrCache>
-                <c:ptCount val="7"/>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>24-Sep</c:v>
-                  </c:pt>
-                  <c:pt idx="1">
-                    <c:v>5-Oct</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>26-Oct</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>17-Nov</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>24-Sep</c:v>
-                  </c:pt>
-                  <c:pt idx="5">
-                    <c:v>5-Oct</c:v>
-                  </c:pt>
-                  <c:pt idx="6">
-                    <c:v>26-Oct</c:v>
-                  </c:pt>
-                </c:lvl>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>SVM</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>RFO</c:v>
-                  </c:pt>
-                </c:lvl>
-              </c:multiLvlStrCache>
-            </c:multiLvlStrRef>
-          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'08-30 Analysis'!$B$21:$H$21</c:f>
+              <c:f>'08-30 Analysis'!$B$23:$H$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -437,7 +733,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'08-30 Analysis'!$A$22</c:f>
+              <c:f>'08-30 Analysis'!$A$24</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -456,48 +752,9 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:multiLvlStrRef>
-              <c:f>'08-30 Analysis'!$B$1:$H$19</c:f>
-              <c:multiLvlStrCache>
-                <c:ptCount val="7"/>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>24-Sep</c:v>
-                  </c:pt>
-                  <c:pt idx="1">
-                    <c:v>5-Oct</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>26-Oct</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>17-Nov</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>24-Sep</c:v>
-                  </c:pt>
-                  <c:pt idx="5">
-                    <c:v>5-Oct</c:v>
-                  </c:pt>
-                  <c:pt idx="6">
-                    <c:v>26-Oct</c:v>
-                  </c:pt>
-                </c:lvl>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>SVM</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>RFO</c:v>
-                  </c:pt>
-                </c:lvl>
-              </c:multiLvlStrCache>
-            </c:multiLvlStrRef>
-          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'08-30 Analysis'!$B$22:$H$22</c:f>
+              <c:f>'08-30 Analysis'!$B$24:$H$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -551,7 +808,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="d\-mmm" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -768,6 +1025,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -1271,20 +1568,564 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1238250</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>295275</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1219200</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C6D0D7F6-F8EF-B1FA-19D0-9921D1911499}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1310,10 +2151,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1579,11 +2416,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.7109375" customWidth="1"/>
     <col min="4" max="4" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
@@ -1597,430 +2434,77 @@
     <col min="13" max="13" width="27.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="H1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="N1" t="s">
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2">
+        <v>205</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B3" s="2">
+        <v>26</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="2">
-        <v>0.84</v>
-      </c>
-      <c r="C3">
-        <v>0.84</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.8</v>
-      </c>
-      <c r="E3" s="2">
-        <v>0.82</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0.47</v>
-      </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2">
-        <v>0.84</v>
-      </c>
-      <c r="I3" s="2">
-        <v>0.93</v>
-      </c>
-      <c r="J3" s="2"/>
-      <c r="M3">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="E4" s="2">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0.61</v>
-      </c>
+      <c r="B4" s="2">
+        <v>16</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0.91</v>
-      </c>
-      <c r="M4">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0.68</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0.8</v>
-      </c>
-      <c r="E5" s="2">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0.55000000000000004</v>
-      </c>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="2">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0.9</v>
-      </c>
-      <c r="M5">
-        <v>0.92</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6">
-        <v>0.26</v>
-      </c>
-      <c r="C6">
-        <v>0.43</v>
-      </c>
-      <c r="E6">
-        <v>0.27</v>
-      </c>
-      <c r="F6">
-        <v>0.66</v>
-      </c>
-      <c r="H6">
-        <v>0.26</v>
-      </c>
-      <c r="I6">
-        <v>0.08</v>
-      </c>
-      <c r="M6">
-        <v>7.0000000000000007E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>0.46</v>
-      </c>
-      <c r="C7">
-        <v>0.59</v>
-      </c>
-      <c r="E7">
-        <v>0.47</v>
-      </c>
-      <c r="F7">
-        <v>1.06</v>
-      </c>
-      <c r="H7">
-        <v>0.46</v>
-      </c>
-      <c r="I7">
-        <v>0.15</v>
-      </c>
-      <c r="M7">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>-0.32</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>-0.62</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>0.75</v>
-      </c>
-      <c r="M8">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9">
-        <v>0.83</v>
-      </c>
-      <c r="C9">
-        <v>0.65</v>
-      </c>
-      <c r="E9">
-        <v>0.82</v>
-      </c>
-      <c r="F9">
-        <v>0.53</v>
-      </c>
-      <c r="H9">
-        <v>0.83</v>
-      </c>
-      <c r="I9">
-        <v>0.94</v>
-      </c>
-      <c r="M9">
-        <v>0.94</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10">
-        <v>0.84</v>
-      </c>
-      <c r="C10">
-        <v>0.65</v>
-      </c>
-      <c r="E10">
-        <v>0.82</v>
-      </c>
-      <c r="F10">
-        <v>0.53</v>
-      </c>
-      <c r="H10">
-        <v>0.84</v>
-      </c>
-      <c r="I10">
-        <v>0.65</v>
-      </c>
-      <c r="M10">
-        <v>0.53</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="M13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="M14">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="M16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>22</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>23</v>
-      </c>
-      <c r="M18">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>24</v>
-      </c>
-      <c r="M19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>25</v>
-      </c>
-      <c r="M20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>26</v>
-      </c>
-      <c r="M21">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>27</v>
-      </c>
-      <c r="M22">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>28</v>
-      </c>
-      <c r="M23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>29</v>
-      </c>
-      <c r="M24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>30</v>
-      </c>
-      <c r="M25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>31</v>
-      </c>
-      <c r="M26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>32</v>
-      </c>
-      <c r="M27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>33</v>
-      </c>
-      <c r="M28">
-        <v>0</v>
-      </c>
+      <c r="H5" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31B271D7-5147-414E-9D6E-4A27129EAAD6}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D5AA18C-A5F0-4069-B351-4AEFF0D48C38}">
-  <dimension ref="A1:I45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I47"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
@@ -2031,15 +2515,15 @@
     <col min="9" max="9" width="7.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="B2" s="1">
         <v>45193</v>
       </c>
@@ -2065,7 +2549,10 @@
         <v>45247</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9">
+      <c r="A3" s="3" t="s">
+        <v>7</v>
+      </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -2075,7 +2562,10 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -2085,7 +2575,10 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -2095,7 +2588,10 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -2105,7 +2601,10 @@
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2115,7 +2614,10 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -2125,7 +2627,10 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -2135,7 +2640,10 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -2145,9 +2653,9 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>35</v>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>12</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -2158,7 +2666,10 @@
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9">
+      <c r="A12" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -2168,349 +2679,353 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19">
+        <v>0.83699999999999997</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20">
+        <v>0.83699999999999997</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22">
+        <v>0.26</v>
+      </c>
+      <c r="C22">
+        <v>0.35</v>
+      </c>
+      <c r="D22">
+        <v>0.36</v>
+      </c>
+      <c r="E22">
+        <v>0.88</v>
+      </c>
+      <c r="F22">
+        <v>0.33</v>
+      </c>
+      <c r="G22">
+        <v>0.96</v>
+      </c>
+      <c r="H22">
+        <v>0.96</v>
+      </c>
+      <c r="I22">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23">
+        <v>0.24</v>
+      </c>
+      <c r="C23">
+        <v>0.16</v>
+      </c>
+      <c r="D23">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="E23">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0.93</v>
+      </c>
+      <c r="H23">
+        <v>0.95</v>
+      </c>
+      <c r="I23">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0.78</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>0.9</v>
+      </c>
+      <c r="H24">
+        <v>0.87</v>
+      </c>
+      <c r="I24">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="C25">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E25">
+        <v>0.38</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="I25">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" t="s">
         <v>9</v>
       </c>
-      <c r="B20">
-        <v>0.26</v>
-      </c>
-      <c r="C20">
-        <v>0.35</v>
-      </c>
-      <c r="D20">
-        <v>0.36</v>
-      </c>
-      <c r="E20">
-        <v>0.88</v>
-      </c>
-      <c r="F20">
+      <c r="B26">
+        <v>1.96</v>
+      </c>
+      <c r="C26">
+        <v>1.88</v>
+      </c>
+      <c r="E26">
+        <v>0.53</v>
+      </c>
+      <c r="F26">
+        <v>1.66</v>
+      </c>
+      <c r="I26">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>10</v>
+      </c>
+      <c r="B27">
+        <v>-1.29</v>
+      </c>
+      <c r="C27">
+        <v>-0.98</v>
+      </c>
+      <c r="E27">
+        <v>-0.26</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28">
+        <v>0.25</v>
+      </c>
+      <c r="C28">
+        <v>0.27</v>
+      </c>
+      <c r="E28">
+        <v>0.68</v>
+      </c>
+      <c r="F28">
         <v>0.33</v>
       </c>
-      <c r="G20">
+      <c r="I28">
         <v>0.96</v>
       </c>
-      <c r="H20">
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29">
+        <v>0.25</v>
+      </c>
+      <c r="C29">
+        <v>0.27</v>
+      </c>
+      <c r="E29">
+        <v>0.68</v>
+      </c>
+      <c r="F29">
+        <v>0.25</v>
+      </c>
+      <c r="I29">
         <v>0.96</v>
       </c>
-      <c r="I20">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21">
-        <v>0.24</v>
-      </c>
-      <c r="C21">
-        <v>0.16</v>
-      </c>
-      <c r="D21">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="E21">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="F21">
-        <v>0</v>
-      </c>
-      <c r="G21">
-        <v>0.93</v>
-      </c>
-      <c r="H21">
-        <v>0.95</v>
-      </c>
-      <c r="I21">
-        <v>0.93</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>11</v>
-      </c>
-      <c r="B22">
-        <v>0</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22">
-        <v>0.78</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-      <c r="G22">
-        <v>0.9</v>
-      </c>
-      <c r="H22">
-        <v>0.87</v>
-      </c>
-      <c r="I22">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B23">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="C23">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="E23">
-        <v>0.38</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="I23">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24">
-        <v>1.96</v>
-      </c>
-      <c r="C24">
-        <v>1.88</v>
-      </c>
-      <c r="E24">
-        <v>0.53</v>
-      </c>
-      <c r="F24">
-        <v>1.66</v>
-      </c>
-      <c r="I24">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>14</v>
-      </c>
-      <c r="B25">
-        <v>-1.29</v>
-      </c>
-      <c r="C25">
-        <v>-0.98</v>
-      </c>
-      <c r="E25">
-        <v>-0.26</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-      <c r="I25">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" t="s">
         <v>15</v>
       </c>
-      <c r="B26">
-        <v>0.25</v>
-      </c>
-      <c r="C26">
-        <v>0.27</v>
-      </c>
-      <c r="E26">
-        <v>0.68</v>
-      </c>
-      <c r="F26">
-        <v>0.33</v>
-      </c>
-      <c r="I26">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" t="s">
         <v>16</v>
       </c>
-      <c r="B27">
-        <v>0.25</v>
-      </c>
-      <c r="C27">
-        <v>0.27</v>
-      </c>
-      <c r="E27">
-        <v>0.68</v>
-      </c>
-      <c r="F27">
-        <v>0.25</v>
-      </c>
-      <c r="I27">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="37" spans="1:1">
+      <c r="A37" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="38" spans="1:1">
+      <c r="A38" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="39" spans="1:1">
+      <c r="A39" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="40" spans="1:1">
+      <c r="A40" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="41" spans="1:1">
+      <c r="A41" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="42" spans="1:1">
+      <c r="A42" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="43" spans="1:1">
+      <c r="A43" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="44" spans="1:1">
+      <c r="A44" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="45" spans="1:1">
+      <c r="A45" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="46" spans="1:1">
+      <c r="A46" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="47" spans="1:1">
+      <c r="A47" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2520,30 +3035,30 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA01A254-30FA-4066-BC2B-BE8C98A6CE0D}">
   <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="B1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B3">
         <v>0.23</v>
@@ -2552,9 +3067,9 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>0.28999999999999998</v>
@@ -2563,9 +3078,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B5">
         <v>0.26</v>
@@ -2574,9 +3089,9 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>0.71</v>
@@ -2585,9 +3100,9 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>1.1599999999999999</v>
@@ -2596,9 +3111,9 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>-0.54</v>
@@ -2607,9 +3122,9 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>0.51</v>
@@ -2618,9 +3133,9 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>0.51</v>
@@ -2629,89 +3144,89 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="27" spans="1:1">
+      <c r="A27" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2719,30 +3234,30 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04300482-AF1D-4DE0-B0C9-9A57AF676E66}">
   <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" customWidth="1"/>
     <col min="4" max="4" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="B1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B3">
         <v>0.23</v>
@@ -2751,9 +3266,9 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>0.28999999999999998</v>
@@ -2762,9 +3277,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B5">
         <v>0.26</v>
@@ -2773,9 +3288,9 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>0.71</v>
@@ -2784,9 +3299,9 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>1.1599999999999999</v>
@@ -2795,9 +3310,9 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>-0.54</v>
@@ -2806,9 +3321,9 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>0.51</v>
@@ -2817,9 +3332,9 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>0.51</v>
@@ -2828,89 +3343,89 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="27" spans="1:1">
+      <c r="A27" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generating vegetation indices using QUAC calibrated imagery.
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26501"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26502"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sluedu-my.sharepoint.com/personal/felipe_lopes_slu_edu/Documents/Desktop/Repos/plant-disease-prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="508" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5390C6E-E83E-4D55-8EAB-F63804077374}"/>
+  <xr:revisionPtr revIDLastSave="544" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C05425BE-44DA-4600-99D6-A0FB60841874}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall Analysis" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="35">
   <si>
     <t>Dataset</t>
   </si>
@@ -62,6 +62,9 @@
     <t>RFO</t>
   </si>
   <si>
+    <t>CNN</t>
+  </si>
+  <si>
     <t>SYNTHETICALLY BALANCED</t>
   </si>
   <si>
@@ -81,6 +84,9 @@
   </si>
   <si>
     <t>UNBALANCED</t>
+  </si>
+  <si>
+    <t>Validation</t>
   </si>
   <si>
     <t>OVERSAMPLED</t>
@@ -613,7 +619,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'08-30 Analysis'!$A$22</c:f>
+              <c:f>'08-30 Analysis'!$A$24</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -634,7 +640,7 @@
           <c:invertIfNegative val="0"/>
           <c:val>
             <c:numRef>
-              <c:f>'08-30 Analysis'!$B$22:$H$22</c:f>
+              <c:f>'08-30 Analysis'!$B$24:$H$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -673,7 +679,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'08-30 Analysis'!$A$23</c:f>
+              <c:f>'08-30 Analysis'!$A$25</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -694,7 +700,7 @@
           <c:invertIfNegative val="0"/>
           <c:val>
             <c:numRef>
-              <c:f>'08-30 Analysis'!$B$23:$H$23</c:f>
+              <c:f>'08-30 Analysis'!$B$25:$H$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -733,7 +739,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'08-30 Analysis'!$A$24</c:f>
+              <c:f>'08-30 Analysis'!$A$26</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -754,7 +760,7 @@
           <c:invertIfNegative val="0"/>
           <c:val>
             <c:numRef>
-              <c:f>'08-30 Analysis'!$B$24:$H$24</c:f>
+              <c:f>'08-30 Analysis'!$B$26:$H$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -2116,16 +2122,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>314325</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2501,7 +2507,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D5AA18C-A5F0-4069-B351-4AEFF0D48C38}">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -2515,15 +2521,18 @@
     <col min="9" max="9" width="7.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:13">
       <c r="B1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="B2" s="1">
         <v>45193</v>
       </c>
@@ -2548,10 +2557,22 @@
       <c r="I2" s="1">
         <v>45247</v>
       </c>
-    </row>
-    <row r="3" spans="1:9">
+      <c r="J2" s="1">
+        <v>45193</v>
+      </c>
+      <c r="K2" s="1">
+        <v>45204</v>
+      </c>
+      <c r="L2" s="1">
+        <v>45225</v>
+      </c>
+      <c r="M2" s="1">
+        <v>45247</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -2562,7 +2583,7 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2575,7 +2596,7 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2588,7 +2609,7 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -2601,9 +2622,9 @@
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -2614,9 +2635,9 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -2627,9 +2648,9 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -2640,9 +2661,9 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -2653,9 +2674,9 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -2666,10 +2687,7 @@
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
     </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="3" t="s">
-        <v>13</v>
-      </c>
+    <row r="12" spans="1:13">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -2679,353 +2697,433 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
     </row>
-    <row r="13" spans="1:9">
-      <c r="A13" t="s">
+    <row r="13" spans="1:13">
+      <c r="A13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" t="s">
         <v>4</v>
-      </c>
-      <c r="B13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" t="s">
-        <v>3</v>
       </c>
       <c r="B14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:9">
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16" t="s">
         <v>2</v>
       </c>
-      <c r="B15">
-        <v>0.84</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" t="s">
-        <v>8</v>
-      </c>
       <c r="B16">
-        <v>0.26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+        <v>0.83699999999999997</v>
+      </c>
+      <c r="F16">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="J16">
+        <v>0.80600000000000005</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
       <c r="A17" t="s">
         <v>9</v>
       </c>
       <c r="B17">
-        <v>0.48</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+        <v>0.27</v>
+      </c>
+      <c r="F17">
+        <v>0.32</v>
+      </c>
+      <c r="J17">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
       <c r="A18" t="s">
         <v>10</v>
       </c>
       <c r="B18">
-        <v>-0.17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+        <v>0.48</v>
+      </c>
+      <c r="F18">
+        <v>0.59</v>
+      </c>
+      <c r="J18">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
       <c r="A19" t="s">
         <v>11</v>
       </c>
       <c r="B19">
-        <v>0.83699999999999997</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+        <v>-0.17</v>
+      </c>
+      <c r="F19">
+        <v>-0.43</v>
+      </c>
+      <c r="J19">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
       <c r="A20" t="s">
         <v>12</v>
       </c>
       <c r="B20">
         <v>0.83699999999999997</v>
       </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-    </row>
-    <row r="22" spans="1:9">
+      <c r="F20">
+        <v>0.81</v>
+      </c>
+      <c r="J20">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21">
+        <v>0.83699999999999997</v>
+      </c>
+      <c r="F21">
+        <v>0.81</v>
+      </c>
+      <c r="J21">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
       <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22">
+        <v>0.8</v>
+      </c>
+      <c r="F22">
+        <v>0.77</v>
+      </c>
+      <c r="J22">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" t="s">
         <v>4</v>
       </c>
-      <c r="B22">
+      <c r="B24">
         <v>0.26</v>
       </c>
-      <c r="C22">
+      <c r="C24">
         <v>0.35</v>
       </c>
-      <c r="D22">
+      <c r="D24">
         <v>0.36</v>
       </c>
-      <c r="E22">
+      <c r="E24">
         <v>0.88</v>
       </c>
-      <c r="F22">
+      <c r="F24">
         <v>0.33</v>
       </c>
-      <c r="G22">
+      <c r="G24">
         <v>0.96</v>
       </c>
-      <c r="H22">
+      <c r="H24">
         <v>0.96</v>
       </c>
-      <c r="I22">
+      <c r="I24">
         <v>0.9</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
-      <c r="A23" t="s">
+    <row r="25" spans="1:10">
+      <c r="A25" t="s">
         <v>3</v>
       </c>
-      <c r="B23">
+      <c r="B25">
         <v>0.24</v>
       </c>
-      <c r="C23">
+      <c r="C25">
         <v>0.16</v>
       </c>
-      <c r="D23">
+      <c r="D25">
         <v>0.55000000000000004</v>
       </c>
-      <c r="E23">
+      <c r="E25">
         <v>0.57999999999999996</v>
       </c>
-      <c r="F23">
+      <c r="F25">
         <v>0</v>
       </c>
-      <c r="G23">
+      <c r="G25">
         <v>0.93</v>
       </c>
-      <c r="H23">
+      <c r="H25">
         <v>0.95</v>
       </c>
-      <c r="I23">
+      <c r="I25">
         <v>0.93</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
-      <c r="A24" t="s">
+    <row r="26" spans="1:10">
+      <c r="A26" t="s">
         <v>2</v>
       </c>
-      <c r="B24">
+      <c r="B26">
         <v>0</v>
       </c>
-      <c r="C24">
+      <c r="C26">
         <v>0</v>
       </c>
-      <c r="D24">
+      <c r="D26">
         <v>0</v>
       </c>
-      <c r="E24">
+      <c r="E26">
         <v>0.78</v>
       </c>
-      <c r="F24">
+      <c r="F26">
         <v>0</v>
       </c>
-      <c r="G24">
+      <c r="G26">
         <v>0.9</v>
       </c>
-      <c r="H24">
+      <c r="H26">
         <v>0.87</v>
       </c>
-      <c r="I24">
+      <c r="I26">
         <v>0.96</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
-      <c r="A25" t="s">
-        <v>8</v>
-      </c>
-      <c r="B25">
+    <row r="27" spans="1:10">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27">
         <v>1.1499999999999999</v>
       </c>
-      <c r="C25">
+      <c r="C27">
         <v>1.1000000000000001</v>
       </c>
-      <c r="E25">
+      <c r="E27">
         <v>0.38</v>
       </c>
-      <c r="F25">
+      <c r="F27">
         <v>1</v>
       </c>
-      <c r="I25">
+      <c r="I27">
         <v>0.05</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
-      <c r="A26" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26">
+    <row r="28" spans="1:10">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28">
         <v>1.96</v>
       </c>
-      <c r="C26">
+      <c r="C28">
         <v>1.88</v>
       </c>
-      <c r="E26">
+      <c r="E28">
         <v>0.53</v>
       </c>
-      <c r="F26">
+      <c r="F28">
         <v>1.66</v>
       </c>
-      <c r="I26">
+      <c r="I28">
         <v>0.09</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
-      <c r="A27" t="s">
-        <v>10</v>
-      </c>
-      <c r="B27">
+    <row r="29" spans="1:10">
+      <c r="A29" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29">
         <v>-1.29</v>
       </c>
-      <c r="C27">
+      <c r="C29">
         <v>-0.98</v>
       </c>
-      <c r="E27">
+      <c r="E29">
         <v>-0.26</v>
       </c>
-      <c r="F27">
+      <c r="F29">
         <v>0</v>
       </c>
-      <c r="I27">
+      <c r="I29">
         <v>0.85</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
-      <c r="A28" t="s">
-        <v>11</v>
-      </c>
-      <c r="B28">
+    <row r="30" spans="1:10">
+      <c r="A30" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30">
         <v>0.25</v>
       </c>
-      <c r="C28">
+      <c r="C30">
         <v>0.27</v>
       </c>
-      <c r="E28">
+      <c r="E30">
         <v>0.68</v>
       </c>
-      <c r="F28">
+      <c r="F30">
         <v>0.33</v>
       </c>
-      <c r="I28">
+      <c r="I30">
         <v>0.96</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
-      <c r="A29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B29">
+    <row r="31" spans="1:10">
+      <c r="A31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31">
         <v>0.25</v>
       </c>
-      <c r="C29">
+      <c r="C31">
         <v>0.27</v>
       </c>
-      <c r="E29">
+      <c r="E31">
         <v>0.68</v>
       </c>
-      <c r="F29">
+      <c r="F31">
         <v>0.25</v>
       </c>
-      <c r="I29">
+      <c r="I31">
         <v>0.96</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
-      <c r="A31" t="s">
+    <row r="32" spans="1:10">
+      <c r="A32" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9">
-      <c r="A32" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1">
-      <c r="A33" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -3053,7 +3151,7 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -3091,7 +3189,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6">
         <v>0.71</v>
@@ -3102,7 +3200,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7">
         <v>1.1599999999999999</v>
@@ -3113,7 +3211,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8">
         <v>-0.54</v>
@@ -3124,7 +3222,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9">
         <v>0.51</v>
@@ -3135,7 +3233,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B10">
         <v>0.51</v>
@@ -3146,87 +3244,87 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -3252,7 +3350,7 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -3290,7 +3388,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6">
         <v>0.71</v>
@@ -3301,7 +3399,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7">
         <v>1.1599999999999999</v>
@@ -3312,7 +3410,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8">
         <v>-0.54</v>
@@ -3323,7 +3421,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9">
         <v>0.51</v>
@@ -3334,7 +3432,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B10">
         <v>0.51</v>
@@ -3345,87 +3443,87 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Splitting the feature extraction and feature-based classification tasks.
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sluedu-my.sharepoint.com/personal/felipe_lopes_slu_edu/Documents/Desktop/Repos/plant-disease-prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="544" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C05425BE-44DA-4600-99D6-A0FB60841874}"/>
+  <xr:revisionPtr revIDLastSave="604" documentId="11_F25DC773A252ABDACC1048F7011D70BA5BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C43BC295-B6F3-47A4-A6CE-EA0BAD17B807}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,8 +38,35 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={E20E007D-84DB-42B0-99BE-7E9A4718ADD0}</author>
+    <author>tc={AD73B99D-99C4-4B4F-8B35-4DE55D973993}</author>
+  </authors>
+  <commentList>
+    <comment ref="A19" authorId="0" shapeId="0" xr:uid="{E20E007D-84DB-42B0-99BE-7E9A4718ADD0}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not suitable for classification problems</t>
+      </text>
+    </comment>
+    <comment ref="F22" authorId="1" shapeId="0" xr:uid="{AD73B99D-99C4-4B4F-8B35-4DE55D973993}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    {'n_estimators': 100, 'max_features': 5, 'sqrt', 'max_depth': 4, 'criterion': 'gini'}</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="36">
   <si>
     <t>Dataset</t>
   </si>
@@ -86,10 +113,13 @@
     <t>UNBALANCED</t>
   </si>
   <si>
+    <t>K-Fold Validation (10)</t>
+  </si>
+  <si>
+    <t>OVERSAMPLED</t>
+  </si>
+  <si>
     <t>Validation</t>
-  </si>
-  <si>
-    <t>OVERSAMPLED</t>
   </si>
   <si>
     <t>Feature Importance</t>
@@ -167,12 +197,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -187,11 +223,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -538,459 +575,6 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Oversampled Dataset</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'08-30 Analysis'!$A$24</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Healthy</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:val>
-            <c:numRef>
-              <c:f>'08-30 Analysis'!$B$24:$H$24</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>0.26</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.35</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.36</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.88</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.33</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.96</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.96</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4E54-426B-BD4E-28F324D14057}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'08-30 Analysis'!$A$25</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Unhealthy</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:val>
-            <c:numRef>
-              <c:f>'08-30 Analysis'!$B$25:$H$25</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>0.24</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.16</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.55000000000000004</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.57999999999999996</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.93</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.95</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-4E54-426B-BD4E-28F324D14057}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'08-30 Analysis'!$A$26</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Mild</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent3"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:val>
-            <c:numRef>
-              <c:f>'08-30 Analysis'!$B$26:$H$26</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.78</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.9</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.87</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-4E54-426B-BD4E-28F324D14057}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
-        <c:axId val="1395168871"/>
-        <c:axId val="1767486695"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="1395168871"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="d\-mmm" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1767486695"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="1767486695"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="1"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1395168871"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1031,550 +615,7 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2118,45 +1159,10 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Gráfico 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3726665D-7B59-1CA0-352B-1E3112FD176C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Felipe Lopes" id="{4DDFB9EB-F837-42D9-9956-3D425AF4D894}" userId="S::felipe.lopes@slu.edu::4bdb0b5e-4475-4c16-a556-21f4cfdb5421" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2420,6 +1426,17 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A19" dT="2023-05-10T19:33:29.06" personId="{4DDFB9EB-F837-42D9-9956-3D425AF4D894}" id="{E20E007D-84DB-42B0-99BE-7E9A4718ADD0}">
+    <text>Not suitable for classification problems</text>
+  </threadedComment>
+  <threadedComment ref="F22" dT="2023-05-09T21:49:08.52" personId="{4DDFB9EB-F837-42D9-9956-3D425AF4D894}" id="{AD73B99D-99C4-4B4F-8B35-4DE55D973993}">
+    <text>{'n_estimators': 100, 'max_features': 5, 'sqrt', 'max_depth': 4, 'criterion': 'gini'}</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J5"/>
@@ -2506,7 +1523,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D5AA18C-A5F0-4069-B351-4AEFF0D48C38}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D5AA18C-A5F0-4069-B351-4AEFF0D48C38}">
   <dimension ref="A1:M50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2743,100 +1760,100 @@
         <v>2</v>
       </c>
       <c r="B16">
-        <v>0.83699999999999997</v>
+        <v>0.82599999999999996</v>
       </c>
       <c r="F16">
-        <v>0.83299999999999996</v>
+        <v>0.8</v>
       </c>
       <c r="J16">
-        <v>0.80600000000000005</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" t="s">
         <v>9</v>
       </c>
       <c r="B17">
-        <v>0.27</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="F17">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="J17">
-        <v>0.44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" t="s">
         <v>10</v>
       </c>
       <c r="B18">
-        <v>0.48</v>
+        <v>0.49</v>
       </c>
       <c r="F18">
-        <v>0.59</v>
+        <v>0.64</v>
       </c>
       <c r="J18">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10">
-      <c r="A19" t="s">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B19">
-        <v>-0.17</v>
-      </c>
-      <c r="F19">
+      <c r="B19" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4">
         <v>-0.43</v>
       </c>
-      <c r="J19">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10">
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4">
+        <v>-0.21</v>
+      </c>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+    </row>
+    <row r="20" spans="1:13">
       <c r="A20" t="s">
         <v>12</v>
       </c>
       <c r="B20">
-        <v>0.83699999999999997</v>
+        <v>0.82599999999999996</v>
       </c>
       <c r="F20">
-        <v>0.81</v>
+        <v>0.78</v>
       </c>
       <c r="J20">
-        <v>0.76</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
       <c r="A21" t="s">
         <v>13</v>
       </c>
-      <c r="B21">
-        <v>0.83699999999999997</v>
-      </c>
-      <c r="F21">
-        <v>0.81</v>
-      </c>
-      <c r="J21">
-        <v>0.83</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
+    </row>
+    <row r="22" spans="1:13">
       <c r="A22" t="s">
         <v>15</v>
       </c>
       <c r="B22">
-        <v>0.8</v>
+        <v>0.81399999999999995</v>
       </c>
       <c r="F22">
-        <v>0.77</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="J22">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10">
+        <v>0.66700000000000004</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" s="3" t="s">
         <v>16</v>
       </c>
@@ -2849,287 +1866,140 @@
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:13">
       <c r="A24" t="s">
         <v>4</v>
       </c>
-      <c r="B24">
-        <v>0.26</v>
-      </c>
-      <c r="C24">
-        <v>0.35</v>
-      </c>
-      <c r="D24">
-        <v>0.36</v>
-      </c>
-      <c r="E24">
-        <v>0.88</v>
-      </c>
-      <c r="F24">
-        <v>0.33</v>
-      </c>
-      <c r="G24">
-        <v>0.96</v>
-      </c>
-      <c r="H24">
-        <v>0.96</v>
-      </c>
-      <c r="I24">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10">
+    </row>
+    <row r="25" spans="1:13">
       <c r="A25" t="s">
         <v>3</v>
       </c>
-      <c r="B25">
-        <v>0.24</v>
-      </c>
-      <c r="C25">
-        <v>0.16</v>
-      </c>
-      <c r="D25">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="E25">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-      <c r="G25">
-        <v>0.93</v>
-      </c>
-      <c r="H25">
-        <v>0.95</v>
-      </c>
-      <c r="I25">
-        <v>0.93</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10">
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" t="s">
         <v>2</v>
       </c>
-      <c r="B26">
-        <v>0</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26">
-        <v>0.78</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26">
-        <v>0.9</v>
-      </c>
-      <c r="H26">
-        <v>0.87</v>
-      </c>
-      <c r="I26">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10">
+    </row>
+    <row r="27" spans="1:13">
       <c r="A27" t="s">
         <v>9</v>
       </c>
-      <c r="B27">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="C27">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="E27">
-        <v>0.38</v>
-      </c>
-      <c r="F27">
-        <v>1</v>
-      </c>
-      <c r="I27">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10">
+    </row>
+    <row r="28" spans="1:13">
       <c r="A28" t="s">
         <v>10</v>
       </c>
-      <c r="B28">
-        <v>1.96</v>
-      </c>
-      <c r="C28">
-        <v>1.88</v>
-      </c>
-      <c r="E28">
-        <v>0.53</v>
-      </c>
-      <c r="F28">
-        <v>1.66</v>
-      </c>
-      <c r="I28">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10">
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" t="s">
         <v>11</v>
       </c>
-      <c r="B29">
-        <v>-1.29</v>
-      </c>
-      <c r="C29">
-        <v>-0.98</v>
-      </c>
-      <c r="E29">
-        <v>-0.26</v>
-      </c>
-      <c r="F29">
-        <v>0</v>
-      </c>
-      <c r="I29">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10">
+    </row>
+    <row r="30" spans="1:13">
       <c r="A30" t="s">
         <v>12</v>
       </c>
-      <c r="B30">
-        <v>0.25</v>
-      </c>
-      <c r="C30">
-        <v>0.27</v>
-      </c>
-      <c r="E30">
-        <v>0.68</v>
-      </c>
-      <c r="F30">
-        <v>0.33</v>
-      </c>
-      <c r="I30">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10">
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" t="s">
         <v>13</v>
       </c>
-      <c r="B31">
-        <v>0.25</v>
-      </c>
-      <c r="C31">
-        <v>0.27</v>
-      </c>
-      <c r="E31">
-        <v>0.68</v>
-      </c>
-      <c r="F31">
-        <v>0.25</v>
-      </c>
-      <c r="I31">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10">
+    </row>
+    <row r="32" spans="1:13">
       <c r="A32" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="50" spans="1:1">
       <c r="A50" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3151,7 +2021,7 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -3244,87 +2114,87 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -3350,7 +2220,7 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -3443,87 +2313,87 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>